<commit_message>
P29 L0 pre: remove prompt 28's army-band upkeep; the supply upkeep stays the only upkeep
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015MqzP1WjPjUApjyRzo5SqY
</commit_message>
<xml_diff>
--- a/Docs/ai/Machine_Brigade_AI_Research_applied.xlsx
+++ b/Docs/ai/Machine_Brigade_AI_Research_applied.xlsx
@@ -2968,9 +2968,6 @@
           <t>Thu nhập đầy đủ</t>
         </is>
       </c>
-      <c r="G16" s="29" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="18">
       <c r="A17" s="34" t="inlineStr">
@@ -2993,9 +2990,6 @@
           <t>Bắt đầu giảm nhẹ (thử 0,85–1,0)</t>
         </is>
       </c>
-      <c r="G17" s="29" t="n">
-        <v>0.9</v>
-      </c>
     </row>
     <row r="18" ht="22.35" customHeight="1" s="18">
       <c r="A18" s="34" t="inlineStr">
@@ -3017,9 +3011,6 @@
         <is>
           <t>Khởi điểm 0,80, chỉ là giá trị đầu; mô phỏng thử 0,65–0,95 và đo vòng lặp nhiều quân → ít thu nhập → quân chết → thu nhập tăng</t>
         </is>
-      </c>
-      <c r="G18" s="29" t="n">
-        <v>0.8</v>
       </c>
     </row>
     <row r="19"/>

</xml_diff>